<commit_message>
Group A (non-FS): 93 Brennan cells mapped by name / sibling / Air-Way donor, staged; FS group A needs the 18 per-dash end STEPs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PJcT2926CUEincCxCV1ZSx
</commit_message>
<xml_diff>
--- a/tools/_out/brennancad_20261021/stage/04_DESIGN_TABLES/DesignTable_5406C.xlsx
+++ b/tools/_out/brennancad_20261021/stage/04_DESIGN_TABLES/DesignTable_5406C.xlsx
@@ -888,6 +888,9 @@
           <t>5406-C-24</t>
         </is>
       </c>
+      <c r="B10" t="n">
+        <v>1.54</v>
+      </c>
       <c r="D10" t="n">
         <v>1.72</v>
       </c>
@@ -906,12 +909,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>[A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: THDMAJ_A@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING</t>
+          <t>[A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: THDMAJ_A@DRIVE, L@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>BUILD-MISSING: part exists in OMi catalog but the Air-Way page has no row; needs a second dimensional source | Brennan CAD record 5406-C-24 (PARTcommunity / CADENAS, THDMAJ_A@DRIVE=A1THD; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -24 1.72 (A1, A9: Brennan 5405-24-24 / -32-32 STEPs 1.734 / 2.218 -&gt; nearest Air-Way 1.72 / 2.20)</t>
+          <t>BUILD-MISSING: part exists in OMi catalog but the Air-Way page has no row; needs a second dimensional source | Brennan CAD record 5406-C-24 (PARTcommunity / CADENAS, THDMAJ_A@DRIVE=A1THD, L@DRIVE=L; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -24 1.72 (A1, A9: Brennan 5405-24-24 / -32-32 STEPs 1.734 / 2.218 -&gt; nearest Air-Way 1.72 / 2.20)</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -936,6 +939,9 @@
           <t>5406-C-32</t>
         </is>
       </c>
+      <c r="B11" t="n">
+        <v>1.64</v>
+      </c>
       <c r="D11" t="n">
         <v>2.2</v>
       </c>
@@ -954,12 +960,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>[A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: THDMAJ_A@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING</t>
+          <t>[A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: THDMAJ_A@DRIVE, L@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BUILD-MISSING: part exists in OMi catalog but the Air-Way page has no row; needs a second dimensional source | Brennan CAD record 5406-C-32 (PARTcommunity / CADENAS, THDMAJ_A@DRIVE=A1THD; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -32 2.2 (A1, A9: Brennan 5405-24-24 / -32-32 STEPs 1.734 / 2.218 -&gt; nearest Air-Way 1.72 / 2.20)</t>
+          <t>BUILD-MISSING: part exists in OMi catalog but the Air-Way page has no row; needs a second dimensional source | Brennan CAD record 5406-C-32 (PARTcommunity / CADENAS, THDMAJ_A@DRIVE=A1THD, L@DRIVE=L; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -32 2.2 (A1, A9: Brennan 5405-24-24 / -32-32 STEPs 1.734 / 2.218 -&gt; nearest Air-Way 1.72 / 2.20)</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">

</xml_diff>